<commit_message>
Add Egypt areas layer: seed sheet with entity types, parent links, learned merge
</commit_message>
<xml_diff>
--- a/egypt_governorates.xlsx
+++ b/egypt_governorates.xlsx
@@ -14,6 +14,7 @@
     <sheet name="الشوارع والمناطق (Template)" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="ملاحظات" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="ملاحظات الإصدار الجديد" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="المناطق والأحياء" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -22951,4 +22952,4003 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G130"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>المناطق والأحياء المصرية (Areas / Neighborhoods / Roads / Compounds / Villages)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>بذرة يدوية لمستوى المنطقة (تحت المحافظة والمدينة). كل كيان له معرّف ثابت ونوع كيان وعلاقة بأبيه. تُدمج مع مناطق areas_learned.json عند بناء اللوك أب — المكتسبة تكمل ولا تحذف النوع من البذرة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>entity_type</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>governorate</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>area_name</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>aliases</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>confidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AR0001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>التجمع الأول</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>التجمع 1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AR0002</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>التجمع الثالث</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>التجمع 3</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AR0003</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>التجمع الخامس</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>التجمع 5</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AR0004</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>الرحاب</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AR0005</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>النرجس</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AR0006</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>القطامية</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AR0007</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>النزهة الجديدة</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>AR0008</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>ريتاج</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>AR0009</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>مدينتي</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AR0010</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>سراي القاهرة</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>سراي</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>AR0011</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ماونتن فيو</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ماونتن فيو 3</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>AR0012</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>فالي</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>فاللي</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>AR0013</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>القاهرة الجديدة</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>وادي دجلة</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>AR0014</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>شرق مدينة نصر</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>الحي الثامن</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>AR0015</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>شرق مدينة نصر</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>الحي السابع</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>AR0016</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>شرق مدينة نصر</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>الحي العاشر</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>AR0017</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>شرق مدينة نصر</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>مكرم عبيد</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>AR0018</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>الزاوية الحمراء</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>بركة النصر</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>AR0019</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>الزيتون</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>حلمية الزيتون</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>AR0020</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>الشروق</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>الهايكستب</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>هيكستب</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>AR0021</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>مدينة السلام</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>شرق مدينة السلام</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>AR0022</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>منشأة ناصر</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>AR0023</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>المطرية</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>AR0024</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>شبرا</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>شبرا القاهرة</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>AR0025</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>العتبة</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>العتبه</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>AR0026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>باب اللوق</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>AR0027</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>الحسين</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>AR0028</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>الفسطاط</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>AR0029</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>العباسية</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>AR0030</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>المعادي الجديدة</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>AR0031</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>المعادي القديمة</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>AR0032</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>حدائق المعادي</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>AR0033</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>عرب المعادي</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>AR0034</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>ميدان التحرير</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>التحرير</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>AR0035</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>ميدان رمسيس</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>AR0036</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>العاصمة الإدارية</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>العاصمة</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>AR0037</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>جسر السويس</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AR0038</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>صلاح سالم</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AR0039</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>الطريق الدائري</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>الدائري</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>AR0040</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>كورنيش النيل</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>AR0041</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>شارع رمسيس</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>AR0042</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>شارع الجمهورية</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>AR0043</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>شارع عبد العزيز</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>AR0044</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>شارع قصر النيل</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>AR0045</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>شارع 26 يوليو</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr"/>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>AR0046</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>شارع عباس العقاد</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>عباس العقاد</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>AR0047</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>شارع مصطفى النحاس</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>مصطفى النحاس</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>AR0048</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>طريق النصر</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>AR0049</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>شارع العروبة</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>AR0050</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>كوبري أكتوبر</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>AR0051</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>محور 26 يوليو</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>AR0052</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>الدقي</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>المهندسين</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>AR0053</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>العجوزة</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>كيت كات</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>AR0054</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>الطالبية</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>الزريبة</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>AR0055</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>أكتوبر (مدينة 6 أكتوبر)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>الحي الثاني</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>AR0056</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>أكتوبر (مدينة 6 أكتوبر)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>حدائق أكتوبر</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>AR0057</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>compound</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>أكتوبر (مدينة 6 أكتوبر)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>بالم هيلز أكتوبر</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>بالم هيلز</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>AR0058</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr"/>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>العمرانية</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>AR0059</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr"/>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>المنيب</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>AR0060</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr"/>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>المعتمدية</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>AR0061</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>صفط اللبن</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>AR0062</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ناهيا</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>AR0063</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr"/>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>زنين</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>AR0064</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>ميدان الجيزة</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>AR0065</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>الهرم</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>شارع الهرم</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>AR0066</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>فيصل</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>شارع فيصل</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>AR0067</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>الدقي</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>شارع جامعة الدول العربية</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>AR0068</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>الدقي</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>شارع التحرير</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>AR0069</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>طريق الفيوم</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>AR0070</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>الجيزة</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>محور صفط اللبن</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>AR0071</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>القليوبية</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>بهتيم</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>AR0072</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>القليوبية</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>الخصوص</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>AR0073</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>القليوبية</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>قليوب</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>القلج</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>AR0074</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>كفر عبده</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>AR0075</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>رشدي</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>AR0076</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ستانلي</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>AR0077</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>الحضرة</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>AR0078</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>السيوف</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>AR0079</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>سيدي بشر</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr"/>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>AR0080</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>المكس</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>AR0081</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>أبيس</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>AR0082</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>محطة الرمل</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>AR0083</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr"/>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>الشاطبي</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>AR0084</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>الإبراهيمية</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>الابراهيميه</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>AR0085</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>فلمنج</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>AR0086</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>سبورتنج</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>AR0087</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>سان ستيفانو</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>سنت ستيفانو</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>AR0088</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>زيزينيا</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>AR0089</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>مصطفى كامل</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>AR0090</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>باب شرق</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>AR0091</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>القباري</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>AR0092</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>العامرية</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>AR0093</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr"/>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>رأس التين</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>AR0094</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr"/>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>بحري</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>بحرية</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>AR0095</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>كورنيش الإسكندرية</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>AR0096</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr"/>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>طريق المحمودية</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>AR0097</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>الإسكندرية</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr"/>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>طريق الجيش</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>AR0098</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>البحيرة</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr"/>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>نوبرية</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>النوبارية</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>AR0099</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>سيدي عبد الرحمن</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>AR0100</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>مطروح</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>الساحل الشمالي</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>AR0101</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>دمياط</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr"/>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>عزبة البرج</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>AR0102</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>دمياط</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr"/>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>شطا</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>AR0103</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>الدقهلية</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>المنصورة</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>سندوب</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>AR0104</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>village</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>الدقهلية</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>شربين</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>محلة أنجاق</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>AR0105</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>الدقهلية</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>بلقاس</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>جمصة</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>AR0106</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>كفر الشيخ</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>البرلس (بلطيم)</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>بلطيم</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>AR0107</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>كفر الشيخ</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr"/>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>مصيف بلطيم</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>AR0108</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>village</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>الغربية</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>المحلة الكبرى</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>محلة روح</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>AR0109</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>village</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>المنوفية</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>قويسنا</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>ميت بره</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>AR0110</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>المنوفية</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>السادات</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>المنطقة الثالثة</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>AR0111</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>الشرقية</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>العاشر من رمضان</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>العاشر</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>العاشر من رمضان</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>AR0112</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>البحر الأحمر</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>مدينة الغردقة</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>سقالة</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>AR0113</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>البحر الأحمر</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>مدينة الغردقة</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>دهار</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>AR0114</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>الفيوم</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>قارون</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>AR0115</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>village</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>أسيوط</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>أسيوط</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>نزلة عبداللاه</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>AR0116</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>أسيوط</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>ديروط</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>ديروط الشريف</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>AR0117</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>قنا</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>قنا</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>دندرة</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>AR0118</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>الأقصر</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>الأقصر</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>الكرنك</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr"/>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>AR0119</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>أسوان</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>البسيلي / الرديسية / أبو سمبل وتوشكى (منطقة النوبة)</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>أبو سمبل</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>AR0120</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>طريق مصر إسكندرية الزراعي</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>الطريق الزراعي</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>AR0121</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>طريق مصر إسكندرية الصحراوي</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>الطريق الصحراوي</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>AR0122</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>طريق القاهرة السويس</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>AR0123</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>طريق القاهرة الإسماعيلية</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>AR0124</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr"/>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>طريق بلبيس</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>بلبيس الصحراوي</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>AR0125</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>الطريق الزراعي الشرقي</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>AR0126</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>road</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>القاهرة</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr"/>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>الطريق الصحراوي الشرقي</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>